<commit_message>
created the new supplementary table for length-mass conversions
</commit_message>
<xml_diff>
--- a/plots/Table1.xlsx
+++ b/plots/Table1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elwel\OneDrive\Desktop\aquatic_data\git\BOSCH\plots\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40436072c29b51f3/University of Johannesburg/Post-Doc/Size-Temperature Changes/BOSCH/plots/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{88659EF2-2DA3-42F3-BCE4-279F66F916D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{04DE0419-81FA-4EA8-BF5B-14DD4E7B220E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{04DE0419-81FA-4EA8-BF5B-14DD4E7B220E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1246,89 +1246,89 @@
   </cellStyleXfs>
   <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1665,661 +1665,642 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A59DB2BA-68F3-4EB9-BC92-CF175D50C3B0}">
   <dimension ref="A1:K24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="106.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:11" ht="103.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="E1" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="F1" s="27" t="s">
+      <c r="F1" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="G1" s="27" t="s">
+      <c r="G1" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="I1" s="27" t="s">
+      <c r="I1" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="J1" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="K1" s="26" t="s">
+      <c r="K1" s="17" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="20" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="6"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="18" t="s">
+    <row r="3" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="24"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="I3" s="18" t="s">
+      <c r="I3" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
     </row>
-    <row r="4" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:11" ht="77" x14ac:dyDescent="0.35">
+      <c r="A4" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="J4" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="K4" s="20" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="12"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="8" t="s">
+    <row r="5" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+      <c r="A5" s="25"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
     </row>
-    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="6"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="2" t="s">
+    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="24"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
     </row>
-    <row r="7" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
+    <row r="7" spans="1:11" ht="77" x14ac:dyDescent="0.35">
+      <c r="A7" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="15" t="s">
+      <c r="G7" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="I7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="J7" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="K7" s="13" t="s">
+      <c r="K7" s="20" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="12"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="8" t="s">
+    <row r="8" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+      <c r="A8" s="25"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
+      <c r="J8" s="21"/>
+      <c r="K8" s="21"/>
     </row>
-    <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="6"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="24" t="s">
+    <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="24"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
     </row>
-    <row r="10" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="17" t="s">
+    <row r="10" spans="1:11" ht="77" x14ac:dyDescent="0.35">
+      <c r="A10" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J10" s="13" t="s">
+      <c r="J10" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="K10" s="13" t="s">
+      <c r="K10" s="20" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="6"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="23" t="s">
+    <row r="11" spans="1:11" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="24"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="H11" s="18" t="s">
+      <c r="H11" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="I11" s="18" t="s">
+      <c r="I11" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="22"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J12" s="13" t="s">
+      <c r="J12" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="K12" s="13" t="s">
+      <c r="K12" s="20" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="6"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="18" t="s">
+    <row r="13" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="24"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="H13" s="18" t="s">
+      <c r="H13" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="I13" s="18" t="s">
+      <c r="I13" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
     </row>
-    <row r="14" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="17" t="s">
+    <row r="14" spans="1:11" ht="77" x14ac:dyDescent="0.35">
+      <c r="A14" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="G14" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="H14" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="I14" s="14" t="s">
+      <c r="I14" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="J14" s="10" t="s">
+      <c r="J14" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="K14" s="13" t="s">
+      <c r="K14" s="20" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="12"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="8" t="s">
+    <row r="15" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+      <c r="A15" s="25"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="H15" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="I15" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="J15" s="10" t="s">
+      <c r="J15" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="K15" s="7"/>
+      <c r="K15" s="21"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="12"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="10" t="s">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" s="25"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="K16" s="7"/>
+      <c r="K16" s="21"/>
     </row>
-    <row r="17" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="6"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="18" t="s">
+    <row r="17" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="24"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K17" s="1"/>
+      <c r="K17" s="22"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A18" s="17" t="s">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A18" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I18" s="13" t="s">
+      <c r="I18" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J18" s="13" t="s">
+      <c r="J18" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="K18" s="13" t="s">
+      <c r="K18" s="20" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="6"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="18" t="s">
+    <row r="19" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="24"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G19" s="19" t="s">
+      <c r="G19" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H19" s="18" t="s">
+      <c r="H19" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" s="17" t="s">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I20" s="10" t="s">
+      <c r="I20" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J20" s="13" t="s">
+      <c r="J20" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="K20" s="13" t="s">
+      <c r="K20" s="20" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="6"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="18" t="s">
+    <row r="21" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="24"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="18" t="s">
+      <c r="H21" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="18" t="s">
+      <c r="I21" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
     </row>
-    <row r="22" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
-      <c r="A22" s="17" t="s">
+    <row r="22" spans="1:11" ht="77" x14ac:dyDescent="0.35">
+      <c r="A22" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G22" s="15" t="s">
+      <c r="G22" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H22" s="14" t="s">
+      <c r="H22" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I22" s="14" t="s">
+      <c r="I22" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="J22" s="13" t="s">
+      <c r="J22" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="K22" s="13" t="s">
+      <c r="K22" s="20" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="12"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="10" t="s">
+    <row r="23" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+      <c r="A23" s="25"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="G23" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H23" s="8" t="s">
+      <c r="H23" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I23" s="8" t="s">
+      <c r="I23" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="21"/>
     </row>
-    <row r="24" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="6"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="2" t="s">
+    <row r="24" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="24"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
+      <c r="J24" s="22"/>
+      <c r="K24" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="64">
-    <mergeCell ref="J7:J9"/>
-    <mergeCell ref="K7:K9"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="I4:I6"/>
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="J10:J11"/>
-    <mergeCell ref="J4:J6"/>
-    <mergeCell ref="K4:K6"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="K10:K11"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="D22:D24"/>
-    <mergeCell ref="E22:E24"/>
-    <mergeCell ref="J22:J24"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="J18:J19"/>
     <mergeCell ref="K22:K24"/>
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="B10:B11"/>
@@ -2336,21 +2317,40 @@
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="D18:D19"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="J22:J24"/>
+    <mergeCell ref="J4:J6"/>
+    <mergeCell ref="K4:K6"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="I4:I6"/>
+    <mergeCell ref="J7:J9"/>
+    <mergeCell ref="K7:K9"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="J10:J11"/>
+    <mergeCell ref="K10:K11"/>
     <mergeCell ref="E18:E19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="J18:J19"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="I18:I19"/>
-    <mergeCell ref="K12:K13"/>
-    <mergeCell ref="E14:E17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>